<commit_message>
Revenue map: reference note on components and reports; keep РН wording
- Справка_выручка AdTech_9м2026.docx: the components-to-reports table with
  how each total is built, notes and the supplier-budget block
- standalone xlsx: restore «Реальные направления» / «не-AdTech РН» labels

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TjyVtBMeKRjjZMJmWM6RZp
</commit_message>
<xml_diff>
--- a/Выручка AdTech_9м2026_структура и отчёты.xlsx
+++ b/Выручка AdTech_9м2026_структура и отчёты.xlsx
@@ -779,7 +779,7 @@
       <c r="A6" s="10" t="n"/>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Направления AdTech (без поставщиков М+)</t>
+          <t>Реальные направления AdTech (без поставщиков М+)</t>
         </is>
       </c>
       <c r="C6" s="12">
@@ -2306,7 +2306,7 @@
     <row r="6" ht="30" customHeight="1">
       <c r="B6" s="24" t="inlineStr">
         <is>
-          <t>Направления AdTech: БиП на РН AdTech без поставщиков М+</t>
+          <t>Реальные направления AdTech: БиП на РН AdTech без поставщиков М+</t>
         </is>
       </c>
       <c r="C6" s="25" t="inlineStr">
@@ -2511,7 +2511,7 @@
     <row r="11" ht="30" customHeight="1">
       <c r="B11" s="24" t="inlineStr">
         <is>
-          <t>Доходы на РН других направлений: сделки по данным ДО AdTech</t>
+          <t>Доходы на не-AdTech РН: сделки на РН других направлений по данным ДО AdTech</t>
         </is>
       </c>
       <c r="C11" s="25" t="inlineStr">

</xml_diff>